<commit_message>
Apply deflator for demand response capacity based on share of DR that actually provides when called upon
</commit_message>
<xml_diff>
--- a/InputData/elec/DRC/Demand Response Capacity.xlsx
+++ b/InputData/elec/DRC/Demand Response Capacity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\elec\DRC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\DRC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{726D1944-1CAD-447D-897B-E50B30316ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBF6F814-979D-455D-B8BD-887D64C31E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>Year</t>
   </si>
@@ -144,6 +144,31 @@
   </si>
   <si>
     <t>days and hours correctly in the model.</t>
+  </si>
+  <si>
+    <t>Curtailment Deflator</t>
+  </si>
+  <si>
+    <t>Page 4 (key findings), second bullet</t>
+  </si>
+  <si>
+    <t>California ISO</t>
+  </si>
+  <si>
+    <t>Demand Response Issues and Performance, 2024</t>
+  </si>
+  <si>
+    <t>https://www.caiso.com/documents/demand-response-issues-and-performance-2024-mar-14-2025.pdf</t>
+  </si>
+  <si>
+    <t>We apply a curtailment multiplier to discount the amount of available capacity by the amount of DR that is available</t>
+  </si>
+  <si>
+    <t>on average when called upon. According to CAISO, "on high demand days in the summer, about 70 percent of totaldemand response capacity
+dispatched in real-time reported performing as scheduled"</t>
+  </si>
+  <si>
+    <t>Deflator</t>
   </si>
 </sst>
 </file>
@@ -210,7 +235,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -227,6 +252,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -532,33 +558,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:B37"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="107.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -566,94 +592,135 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" s="2">
         <v>2019</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B20" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B22" s="2">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A21" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A22" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A23" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A25" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A26" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A27" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" s="10" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -669,19 +736,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2019</v>
       </c>
@@ -689,7 +756,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>59000</v>
       </c>
@@ -697,44 +764,54 @@
         <v>198000</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>31</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.75">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>96</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.75">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.75">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>4</v>
       </c>
@@ -751,12 +828,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -860,141 +937,141 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="4">
-        <f>'Data and Calculations'!A3</f>
-        <v>59000</v>
+        <f>'Data and Calculations'!A3*(1-'Data and Calculations'!$A$6)</f>
+        <v>41300</v>
       </c>
       <c r="C2" s="4">
         <f>B2</f>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="D2" s="4">
         <f t="shared" ref="D2:AH2" si="0">C2</f>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="E2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="F2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="G2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="K2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="L2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="M2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="N2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="O2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="P2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="Q2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="R2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="S2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="T2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="U2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="V2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="W2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="X2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="Y2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="Z2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="AA2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="AB2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="AC2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="AD2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="AE2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="AF2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="AG2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
       <c r="AH2" s="4">
         <f t="shared" si="0"/>
-        <v>59000</v>
+        <v>41300</v>
       </c>
     </row>
   </sheetData>
@@ -1008,12 +1085,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1117,141 +1194,141 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:34" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="4">
         <f>C2</f>
-        <v>0</v>
+        <v>12390</v>
       </c>
       <c r="C2" s="4">
-        <f>'Data and Calculations'!A3-'DRC-BDRC'!C2</f>
-        <v>0</v>
+        <f>('Data and Calculations'!A3-'DRC-BDRC'!C2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>12390</v>
       </c>
       <c r="D2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!D1)-'DRC-BDRC'!D2</f>
-        <v>12636.363636363298</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!D1)-'DRC-BDRC'!D2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>21235.454545454308</v>
       </c>
       <c r="E2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!E1)-'DRC-BDRC'!E2</f>
-        <v>25272.727272730321</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!E1)-'DRC-BDRC'!E2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>30080.909090911224</v>
       </c>
       <c r="F2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!F1)-'DRC-BDRC'!F2</f>
-        <v>37909.090909093618</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!F1)-'DRC-BDRC'!F2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>38926.363636365531</v>
       </c>
       <c r="G2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!G1)-'DRC-BDRC'!G2</f>
-        <v>50545.454545456916</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!G1)-'DRC-BDRC'!G2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>47771.818181819835</v>
       </c>
       <c r="H2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!H1)-'DRC-BDRC'!H2</f>
-        <v>63181.818181820214</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!H1)-'DRC-BDRC'!H2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>56617.272727274147</v>
       </c>
       <c r="I2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!I1)-'DRC-BDRC'!I2</f>
-        <v>75818.181818183511</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!I1)-'DRC-BDRC'!I2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>65462.727272728451</v>
       </c>
       <c r="J2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!J1)-'DRC-BDRC'!J2</f>
-        <v>88454.545454546809</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!J1)-'DRC-BDRC'!J2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>74308.181818182755</v>
       </c>
       <c r="K2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!K1)-'DRC-BDRC'!K2</f>
-        <v>101090.90909091011</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!K1)-'DRC-BDRC'!K2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>83153.636363637066</v>
       </c>
       <c r="L2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!L1)-'DRC-BDRC'!L2</f>
-        <v>113727.2727272734</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!L1)-'DRC-BDRC'!L2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>91999.090909091377</v>
       </c>
       <c r="M2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!M1)-'DRC-BDRC'!M2</f>
-        <v>126363.6363636367</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!M1)-'DRC-BDRC'!M2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>100844.54545454569</v>
       </c>
       <c r="N2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!N1)-'DRC-BDRC'!N2</f>
-        <v>139000</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!N1)-'DRC-BDRC'!N2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>109690</v>
       </c>
       <c r="O2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!O1)-'DRC-BDRC'!O2</f>
-        <v>151636.3636363633</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!O1)-'DRC-BDRC'!O2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>118535.4545454543</v>
       </c>
       <c r="P2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!P1)-'DRC-BDRC'!P2</f>
-        <v>164272.72727273032</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!P1)-'DRC-BDRC'!P2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>127380.90909091121</v>
       </c>
       <c r="Q2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!Q1)-'DRC-BDRC'!Q2</f>
-        <v>176909.09090909362</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!Q1)-'DRC-BDRC'!Q2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>136226.36363636554</v>
       </c>
       <c r="R2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!R1)-'DRC-BDRC'!R2</f>
-        <v>189545.45454545692</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!R1)-'DRC-BDRC'!R2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>145071.81818181984</v>
       </c>
       <c r="S2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!S1)-'DRC-BDRC'!S2</f>
-        <v>202181.81818182021</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!S1)-'DRC-BDRC'!S2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>153917.27272727413</v>
       </c>
       <c r="T2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!T1)-'DRC-BDRC'!T2</f>
-        <v>214818.18181818351</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!T1)-'DRC-BDRC'!T2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>162762.72727272846</v>
       </c>
       <c r="U2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!U1)-'DRC-BDRC'!U2</f>
-        <v>227454.54545454681</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!U1)-'DRC-BDRC'!U2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>171608.18181818275</v>
       </c>
       <c r="V2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!V1)-'DRC-BDRC'!V2</f>
-        <v>240090.90909091011</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!V1)-'DRC-BDRC'!V2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>180453.63636363705</v>
       </c>
       <c r="W2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!W1)-'DRC-BDRC'!W2</f>
-        <v>252727.2727272734</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!W1)-'DRC-BDRC'!W2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>189299.09090909138</v>
       </c>
       <c r="X2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!X1)-'DRC-BDRC'!X2</f>
-        <v>265363.6363636367</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!X1)-'DRC-BDRC'!X2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>198144.54545454567</v>
       </c>
       <c r="Y2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!Y1)-'DRC-BDRC'!Y2</f>
-        <v>278000</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!Y1)-'DRC-BDRC'!Y2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>206990</v>
       </c>
       <c r="Z2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!Z1)-'DRC-BDRC'!Z2</f>
-        <v>290636.3636363633</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!Z1)-'DRC-BDRC'!Z2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>215835.4545454543</v>
       </c>
       <c r="AA2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AA1)-'DRC-BDRC'!AA2</f>
-        <v>303272.72727273032</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AA1)-'DRC-BDRC'!AA2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>224680.90909091121</v>
       </c>
       <c r="AB2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AB1)-'DRC-BDRC'!AB2</f>
-        <v>315909.09090909362</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AB1)-'DRC-BDRC'!AB2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>233526.36363636551</v>
       </c>
       <c r="AC2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AC1)-'DRC-BDRC'!AC2</f>
-        <v>328545.45454545692</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AC1)-'DRC-BDRC'!AC2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>242371.81818181984</v>
       </c>
       <c r="AD2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AD1)-'DRC-BDRC'!AD2</f>
-        <v>341181.81818182021</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AD1)-'DRC-BDRC'!AD2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>251217.27272727413</v>
       </c>
       <c r="AE2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AE1)-'DRC-BDRC'!AE2</f>
-        <v>353818.18181818351</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AE1)-'DRC-BDRC'!AE2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>260062.72727272843</v>
       </c>
       <c r="AF2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AF1)-'DRC-BDRC'!AF2</f>
-        <v>366454.54545454681</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AF1)-'DRC-BDRC'!AF2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>268908.18181818275</v>
       </c>
       <c r="AG2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AG1)-'DRC-BDRC'!AG2</f>
-        <v>379090.90909091011</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AG1)-'DRC-BDRC'!AG2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>277753.63636363705</v>
       </c>
       <c r="AH2" s="4">
-        <f>TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AH1)-'DRC-BDRC'!AH2</f>
-        <v>391727.2727272734</v>
+        <f>(TREND('Data and Calculations'!$A$3:$B$3,'Data and Calculations'!$A$2:$B$2,'DRC-PADRC'!AH1)-'DRC-BDRC'!AH2)*(1-'Data and Calculations'!$A$6)</f>
+        <v>286599.09090909135</v>
       </c>
     </row>
   </sheetData>
@@ -1265,13 +1342,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="33.1328125" customWidth="1"/>
-    <col min="2" max="2" width="17.1328125" customWidth="1"/>
+    <col min="1" max="1" width="33.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>15</v>
       </c>
@@ -1279,7 +1356,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>25</v>
       </c>

</xml_diff>